<commit_message>
Added many photos and a new page
</commit_message>
<xml_diff>
--- a/data/travel-captions.xlsx
+++ b/data/travel-captions.xlsx
@@ -4,12 +4,14 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Belgium" sheetId="1" r:id="rId1"/>
-    <sheet name="Greece" sheetId="2" r:id="rId2"/>
-    <sheet name="India" sheetId="3" r:id="rId3"/>
-    <sheet name="Italy" sheetId="4" r:id="rId4"/>
-    <sheet name="Romania" sheetId="5" r:id="rId5"/>
-    <sheet name="United States" sheetId="6" r:id="rId6"/>
-    <sheet name="Vietnam" sheetId="7" r:id="rId7"/>
+    <sheet name="Czechia" sheetId="2" r:id="rId2"/>
+    <sheet name="France" sheetId="3" r:id="rId3"/>
+    <sheet name="Greece" sheetId="4" r:id="rId4"/>
+    <sheet name="India" sheetId="5" r:id="rId5"/>
+    <sheet name="Italy" sheetId="6" r:id="rId6"/>
+    <sheet name="Romania" sheetId="7" r:id="rId7"/>
+    <sheet name="United States" sheetId="8" r:id="rId8"/>
+    <sheet name="Vietnam" sheetId="9" r:id="rId9"/>
   </sheets>
 </workbook>
 </file>
@@ -434,6 +436,180 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B5"/>
+  <cols>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="90.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Photo</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Caption</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>photo 1</v>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>photo 2</v>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>photo 3</v>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>photo 4</v>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B5"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B13"/>
+  <cols>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="90.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Photo</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Caption</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>photo 1</v>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>photo 2</v>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>photo 3</v>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>photo 4</v>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>photo 5</v>
+      </c>
+      <c r="B6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>photo 6</v>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>photo 7</v>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>photo 8</v>
+      </c>
+      <c r="B9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>photo 9</v>
+      </c>
+      <c r="B10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>photo 10</v>
+      </c>
+      <c r="B11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>photo 11</v>
+      </c>
+      <c r="B12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>photo 12</v>
+      </c>
+      <c r="B13" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B13"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B8"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
@@ -511,7 +687,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B7"/>
   <cols>
@@ -582,9 +758,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B13"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="90.83203125" customWidth="1"/>
@@ -603,7 +779,7 @@
         <v>photo 1</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>The Greek myth nerd inside me (and outside) was losing his shit at finally seeing this in person.</v>
       </c>
     </row>
     <row r="3">
@@ -611,7 +787,7 @@
         <v>photo 2</v>
       </c>
       <c r="B3" t="str">
-        <v/>
+        <v>"It is a good life we lead brother"; "Ah, the best"; "May it never change"</v>
       </c>
     </row>
     <row r="4">
@@ -619,7 +795,7 @@
         <v>photo 3</v>
       </c>
       <c r="B4" t="str">
-        <v/>
+        <v>"And may it never change us"</v>
       </c>
     </row>
     <row r="5">
@@ -627,7 +803,7 @@
         <v>photo 4</v>
       </c>
       <c r="B5" t="str">
-        <v/>
+        <v>Hiking on a volcano was not on my bucket list, but it was surreal. Bummer couldn't see the eruption (happened 2 days after we left, smh)</v>
       </c>
     </row>
     <row r="6">
@@ -635,7 +811,7 @@
         <v>photo 5</v>
       </c>
       <c r="B6" t="str">
-        <v/>
+        <v>2026 was the year of having my Assassin's Creed Italy tour.</v>
       </c>
     </row>
     <row r="7">
@@ -643,7 +819,7 @@
         <v>photo 6</v>
       </c>
       <c r="B7" t="str">
-        <v/>
+        <v>Beautiful beautiful Venice...</v>
       </c>
     </row>
     <row r="8">
@@ -670,16 +846,40 @@
         <v/>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>photo 10</v>
+      </c>
+      <c r="B11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>photo 11</v>
+      </c>
+      <c r="B12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>photo 12</v>
+      </c>
+      <c r="B13" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B13"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B13"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="90.83203125" customWidth="1"/>
@@ -733,14 +933,70 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>photo 6</v>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>photo 7</v>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>photo 8</v>
+      </c>
+      <c r="B9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>photo 9</v>
+      </c>
+      <c r="B10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>photo 10</v>
+      </c>
+      <c r="B11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>photo 11</v>
+      </c>
+      <c r="B12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>photo 12</v>
+      </c>
+      <c r="B13" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B13"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B7"/>
   <cols>
@@ -811,9 +1067,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B13"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="90.83203125" customWidth="1"/>
@@ -899,9 +1155,33 @@
         <v/>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>photo 10</v>
+      </c>
+      <c r="B11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>photo 11</v>
+      </c>
+      <c r="B12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>photo 12</v>
+      </c>
+      <c r="B13" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>